<commit_message>
Progressively updating project data tracker.
</commit_message>
<xml_diff>
--- a/QIAL_data_tracker_2019_2026.xlsx
+++ b/QIAL_data_tracker_2019_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rja20/Documents/MATLAB/gunnies/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDC6B3F0-9D5A-EB43-8CD7-520BFBA7A87B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E76E5F50-72B5-B24F-80CC-3E0BD64EDB59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3040" yWindow="4060" windowWidth="38460" windowHeight="20300" activeTab="4" xr2:uid="{BEE67711-3DDE-B344-B789-C2167E37D311}"/>
+    <workbookView xWindow="11120" yWindow="4780" windowWidth="38460" windowHeight="20300" activeTab="4" xr2:uid="{BEE67711-3DDE-B344-B789-C2167E37D311}"/>
   </bookViews>
   <sheets>
     <sheet name="ADRC_human" sheetId="2" r:id="rId1"/>
@@ -18,10 +18,11 @@
     <sheet name="HABS_human" sheetId="1" r:id="rId3"/>
     <sheet name="ADNI_human" sheetId="9" r:id="rId4"/>
     <sheet name="APOEHN_mouse" sheetId="4" r:id="rId5"/>
-    <sheet name="GLP1_mouse" sheetId="5" r:id="rId6"/>
+    <sheet name="T2_masking_invivo_mouse" sheetId="11" r:id="rId6"/>
     <sheet name="Clearance_mouse" sheetId="6" r:id="rId7"/>
-    <sheet name="CVN_mouse" sheetId="7" r:id="rId8"/>
-    <sheet name="C57_mouse" sheetId="8" r:id="rId9"/>
+    <sheet name="GLP1_mouse" sheetId="5" r:id="rId8"/>
+    <sheet name="CVN_mouse" sheetId="7" r:id="rId9"/>
+    <sheet name="C57_mouse" sheetId="8" r:id="rId10"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="431" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="179">
   <si>
     <t>Raw Data</t>
   </si>
@@ -148,9 +149,6 @@
     <t>Main SAMBA work directory ($SAMBA_workdir):</t>
   </si>
   <si>
-    <t>*$SAMBA_workdir is used for brevity, and not an environment variable</t>
-  </si>
-  <si>
     <t>Project: HABS (human)</t>
   </si>
   <si>
@@ -412,9 +410,6 @@
     <t>$DB/Projects/Bruker_Repo/Data/niftis</t>
   </si>
   <si>
-    <t>Renameds (Arunno) niftis</t>
-  </si>
-  <si>
     <t>$DB/Projects/18.abb.11/Analysis</t>
   </si>
   <si>
@@ -431,13 +426,181 @@
   </si>
   <si>
     <t>$SAMBA_workdir/stats_by_region/labels/pre_rigid_native_space/invivoAPOE1/stats</t>
+  </si>
+  <si>
+    <t>Raw Bruker:</t>
+  </si>
+  <si>
+    <t>$MRI/DennisTurner/*/raw</t>
+  </si>
+  <si>
+    <t>$MRI/DennisTurner/*/nii</t>
+  </si>
+  <si>
+    <t>$WORK//DCE_dev/Bruker_radial_recon/Animals_Clearance_Turner_complete_list.xlsx</t>
+  </si>
+  <si>
+    <t>Animal list</t>
+  </si>
+  <si>
+    <t>Project: Brain Clearance (mouse) "Dennis Turner"</t>
+  </si>
+  <si>
+    <t>Project: GLP1 (mouse)</t>
+  </si>
+  <si>
+    <t>$MRI/GLP_1/*/raw</t>
+  </si>
+  <si>
+    <t>Raw from Bruker:</t>
+  </si>
+  <si>
+    <t>$MRI/GLP_1/*/nii</t>
+  </si>
+  <si>
+    <t>$MRI/DennisTurner/all_niis</t>
+  </si>
+  <si>
+    <t>INCOMPLETE BOOKKEEPING/IN PROGRESS</t>
+  </si>
+  <si>
+    <t>Project: C57 (mouse)</t>
+  </si>
+  <si>
+    <t>Project: CVNs (mouse)</t>
+  </si>
+  <si>
+    <t>Initial QA, no coregistration, etc:</t>
+  </si>
+  <si>
+    <t>$MRI/DennisTurner/all_niis/z${runno}/</t>
+  </si>
+  <si>
+    <t>$WORK/DCE_dev/Bruker_radial_recon/</t>
+  </si>
+  <si>
+    <t>www.github.com/andersonion/Bruker_radial_recon</t>
+  </si>
+  <si>
+    <t>CEST:</t>
+  </si>
+  <si>
+    <t>Older batch found in: DB/Projects/18.abb.11/Analysis/mouse_connectomes_080823/mouse_DWI_connectomes</t>
+  </si>
+  <si>
+    <t>2026 Student Work:</t>
+  </si>
+  <si>
+    <t>Project: T2 ML masking (mouse)</t>
+  </si>
+  <si>
+    <t>Main folder:</t>
+  </si>
+  <si>
+    <t>$WORK/skull_stripping</t>
+  </si>
+  <si>
+    <t>Sub folders:</t>
+  </si>
+  <si>
+    <t>T2_prediction</t>
+  </si>
+  <si>
+    <t>T2 input files dated December 2024 (maybe from Hae Sol?)</t>
+  </si>
+  <si>
+    <t>71 manual perfusion masks from 2022 (Nikhil, Jasmine, et al.)</t>
+  </si>
+  <si>
+    <t>perfusion_masks</t>
+  </si>
+  <si>
+    <t>Complete</t>
+  </si>
+  <si>
+    <t>www.github.com/???</t>
+  </si>
+  <si>
+    <t>www.github.com/andersonion/???</t>
+  </si>
+  <si>
+    <t>Aux code 1 (paros): Used here? TBD</t>
+  </si>
+  <si>
+    <t>Main repo (github): *public*</t>
+  </si>
+  <si>
+    <t>Main repo (github): *private, Alex hasn't accepted invite*</t>
+  </si>
+  <si>
+    <t>Aux code 1: (github): *public*</t>
+  </si>
+  <si>
+    <t>$SAMBA_workdir/…</t>
+  </si>
+  <si>
+    <t>Renameds (Arunno) niftis--set this as ''$Analysis"</t>
+  </si>
+  <si>
+    <t>$Analysis/fMRI/fMRI/upgraded_gradients_Duke/</t>
+  </si>
+  <si>
+    <t>T2</t>
+  </si>
+  <si>
+    <t>T1</t>
+  </si>
+  <si>
+    <t>$Analysis/T2_TurboRARE_images/T2_TurboRARE_images/upgraded_gradients_Duke/</t>
+  </si>
+  <si>
+    <t>$Analysis/T1_RARE_images/T1_RARE_images/upgraded_gradients_Duke/</t>
+  </si>
+  <si>
+    <t>raw fMRI</t>
+  </si>
+  <si>
+    <t>/mnt/newStor/paros2/BIAC_munin_dump_20260122/mouse/fMRI_data_packages_for_Nariman/</t>
+  </si>
+  <si>
+    <t>fMRI "packages": fMRI, T1 or T2, maks (usually)</t>
+  </si>
+  <si>
+    <t>raw Perfusion</t>
+  </si>
+  <si>
+    <t>coregistered Perfusion  (4D stack, and average 'p0')</t>
+  </si>
+  <si>
+    <t>$Analysis/Perfusion/Perfusion/; $Analysis/preprocessed_perfusion_data/perfusion_images_Duke_prequench/</t>
+  </si>
+  <si>
+    <t>Perfusion coregistration work</t>
+  </si>
+  <si>
+    <t>$Analysis/pcasl_coreg/pcasl_coregistration_work/</t>
+  </si>
+  <si>
+    <t>$DB/Projects/18.abb.11/Data/unprocessed_bruker_niftis/niftis/*/*pCASL*nii.gz</t>
+  </si>
+  <si>
+    <t>Efficiencies (Perfusion)</t>
+  </si>
+  <si>
+    <t>$Analysis/Efficiencies/Efficiencies/</t>
+  </si>
+  <si>
+    <t>$DB/Projects/18.abb.11/Data/civm_archive/research</t>
+  </si>
+  <si>
+    <t>Raw niftis, btables:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -512,6 +675,21 @@
     <font>
       <sz val="20"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="20"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="20"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -609,7 +787,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -625,7 +803,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -638,6 +816,15 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -663,9 +850,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -703,7 +890,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -809,7 +996,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -951,7 +1138,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -971,16 +1158,16 @@
   <sheetData>
     <row r="1" spans="1:7" ht="31" x14ac:dyDescent="0.35">
       <c r="D1" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="31" x14ac:dyDescent="0.35">
@@ -993,12 +1180,12 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -1010,26 +1197,26 @@
     </row>
     <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B7" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B8" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B9" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -1044,7 +1231,7 @@
         <v>23</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -1060,7 +1247,7 @@
         <v>25</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="15" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -1068,7 +1255,7 @@
         <v>26</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -1076,7 +1263,7 @@
         <v>27</v>
       </c>
       <c r="D16" s="21" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -1084,7 +1271,7 @@
         <v>28</v>
       </c>
       <c r="D17" s="21" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -1092,12 +1279,12 @@
         <v>22</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="19" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B19" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
@@ -1105,13 +1292,13 @@
         <v>3</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C21" s="8"/>
     </row>
     <row r="22" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="24" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
@@ -1163,7 +1350,7 @@
     </row>
     <row r="30" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B30" s="6" t="s">
-        <v>10</v>
+        <v>158</v>
       </c>
       <c r="D30" s="10" t="s">
         <v>13</v>
@@ -1174,6 +1361,237 @@
     <hyperlink ref="D26" r:id="rId1" xr:uid="{8F36A179-6450-B64A-BF84-BA0BF742E49C}"/>
     <hyperlink ref="D28" r:id="rId2" xr:uid="{0C0FD424-EBFC-7347-A47F-F4EE6C751F82}"/>
     <hyperlink ref="D30" r:id="rId3" xr:uid="{32D38EE7-9A59-D143-8027-30B131E6831A}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38B8868B-DAAC-D643-93A0-63D9E1CC5FCA}">
+  <dimension ref="A1:G30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="26" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20.1640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="72.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.83203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="161.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="10.83203125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="31" x14ac:dyDescent="0.35">
+      <c r="D1" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="31" x14ac:dyDescent="0.35">
+      <c r="D2" s="13"/>
+    </row>
+    <row r="3" spans="1:7" ht="31" x14ac:dyDescent="0.35">
+      <c r="A3" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="13"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="14" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+    </row>
+    <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="24" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="24" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D10" s="25"/>
+    </row>
+    <row r="11" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="26"/>
+    </row>
+    <row r="12" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="26" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" s="26" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="26" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15" s="26"/>
+    </row>
+    <row r="16" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D16" s="26"/>
+    </row>
+    <row r="17" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" s="26"/>
+    </row>
+    <row r="18" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D18" s="26" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D19" s="26"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D20" s="25"/>
+    </row>
+    <row r="21" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C21" s="8"/>
+      <c r="D21" s="27"/>
+    </row>
+    <row r="22" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="D22" s="27"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D23" s="25"/>
+    </row>
+    <row r="24" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="28"/>
+    </row>
+    <row r="25" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D25" s="28" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D26" s="29" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D27" s="28" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D28" s="29" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D26" r:id="rId1" xr:uid="{0AA4F660-30A1-BF4B-9DA6-F38F3FB6789B}"/>
+    <hyperlink ref="D28" r:id="rId2" xr:uid="{407F8995-E5CF-F840-9500-E41EF8A0727D}"/>
+    <hyperlink ref="D30" r:id="rId3" xr:uid="{3B0FA85A-A8DF-6D4D-BD35-F91776B09DDE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1197,16 +1615,16 @@
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="13" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="31" x14ac:dyDescent="0.35">
@@ -1218,32 +1636,20 @@
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
     </row>
-    <row r="3" spans="1:7" ht="26" x14ac:dyDescent="0.3">
-      <c r="A3" s="11"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-    </row>
-    <row r="4" spans="1:7" ht="26" x14ac:dyDescent="0.3">
-      <c r="A4" s="11"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-    </row>
-    <row r="5" spans="1:7" ht="26" x14ac:dyDescent="0.3">
-      <c r="A5" s="12"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
+    <row r="3" spans="1:7" s="1" customFormat="1" ht="26" x14ac:dyDescent="0.3">
+      <c r="A3" s="11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" s="1" customFormat="1" ht="26" x14ac:dyDescent="0.3">
+      <c r="A4" s="14" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" s="1" customFormat="1" ht="26" x14ac:dyDescent="0.3">
+      <c r="A5" s="12" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="6" spans="1:7" ht="26" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
@@ -1259,11 +1665,11 @@
     <row r="7" spans="1:7" ht="26" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
@@ -1272,11 +1678,11 @@
     <row r="8" spans="1:7" ht="26" x14ac:dyDescent="0.3">
       <c r="A8" s="16"/>
       <c r="B8" s="16" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C8" s="16"/>
       <c r="D8" s="16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
@@ -1285,11 +1691,11 @@
     <row r="9" spans="1:7" s="17" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
       <c r="B9" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
@@ -1298,11 +1704,11 @@
     <row r="10" spans="1:7" s="17" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
       <c r="B10" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
@@ -1331,11 +1737,11 @@
     <row r="13" spans="1:7" ht="26" x14ac:dyDescent="0.3">
       <c r="A13" s="4"/>
       <c r="B13" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C13" s="4"/>
       <c r="D13" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
@@ -1344,11 +1750,11 @@
     <row r="14" spans="1:7" ht="26" x14ac:dyDescent="0.3">
       <c r="A14" s="4"/>
       <c r="B14" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C14" s="4"/>
       <c r="D14" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
@@ -1357,11 +1763,11 @@
     <row r="15" spans="1:7" ht="26" x14ac:dyDescent="0.3">
       <c r="A15" s="18"/>
       <c r="B15" s="18" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C15" s="18"/>
       <c r="D15" s="18" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E15" s="18"/>
       <c r="F15" s="18"/>
@@ -1370,11 +1776,11 @@
     <row r="16" spans="1:7" s="17" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A16" s="4"/>
       <c r="B16" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C16" s="4"/>
       <c r="D16" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
@@ -1387,7 +1793,7 @@
       </c>
       <c r="C17" s="19"/>
       <c r="D17" s="19" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E17" s="19"/>
       <c r="F17" s="19"/>
@@ -1400,7 +1806,7 @@
       </c>
       <c r="C18" s="4"/>
       <c r="D18" s="23" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
@@ -1413,7 +1819,7 @@
       </c>
       <c r="C19" s="4"/>
       <c r="D19" s="21" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
@@ -1426,7 +1832,7 @@
       </c>
       <c r="C20" s="4"/>
       <c r="D20" s="21" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
@@ -1439,7 +1845,7 @@
       </c>
       <c r="C21" s="4"/>
       <c r="D21" s="21" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
@@ -1452,7 +1858,7 @@
       </c>
       <c r="C22" s="4"/>
       <c r="D22" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
@@ -1481,7 +1887,7 @@
         <v>3</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C25" s="8"/>
       <c r="D25" s="9"/>
@@ -1491,14 +1897,14 @@
     </row>
     <row r="26" spans="1:7" ht="26" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C26" s="9"/>
       <c r="D26" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
@@ -1549,7 +1955,7 @@
     <row r="31" spans="1:7" ht="26" x14ac:dyDescent="0.3">
       <c r="A31" s="6"/>
       <c r="B31" s="6" t="s">
-        <v>8</v>
+        <v>156</v>
       </c>
       <c r="C31" s="6"/>
       <c r="D31" s="10" t="s">
@@ -1575,7 +1981,7 @@
     <row r="33" spans="1:7" ht="26" x14ac:dyDescent="0.3">
       <c r="A33" s="6"/>
       <c r="B33" s="6" t="s">
-        <v>10</v>
+        <v>158</v>
       </c>
       <c r="C33" s="6"/>
       <c r="D33" s="10" t="s">
@@ -1601,7 +2007,7 @@
     <row r="35" spans="1:7" ht="26" x14ac:dyDescent="0.3">
       <c r="A35" s="6"/>
       <c r="B35" s="6" t="s">
-        <v>10</v>
+        <v>158</v>
       </c>
       <c r="C35" s="6"/>
       <c r="D35" s="10" t="s">
@@ -1618,6 +2024,7 @@
     <hyperlink ref="D35" r:id="rId3" xr:uid="{8F4E9AED-317C-BC4E-8FD6-5EB8D63BE6DF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -1636,7 +2043,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="31" x14ac:dyDescent="0.35">
       <c r="D1" s="13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="31" x14ac:dyDescent="0.35">
@@ -1649,12 +2056,12 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -1669,7 +2076,7 @@
         <v>15</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -1703,7 +2110,7 @@
         <v>21</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -1711,7 +2118,7 @@
         <v>29</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -1719,15 +2126,15 @@
         <v>25</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B15" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -1735,15 +2142,15 @@
         <v>27</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B17" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -1757,30 +2164,30 @@
     <row r="19" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
     <row r="20" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B20" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="21" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B21" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D21" s="4" t="s">
         <v>45</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="22" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
     <row r="23" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B23" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D23" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="E23" s="4" t="s">
         <v>48</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="25" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
@@ -1793,30 +2200,30 @@
     <row r="26" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="8"/>
       <c r="B26" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C26" s="8"/>
       <c r="D26" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B27" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="D27" s="9" t="s">
         <v>53</v>
-      </c>
-      <c r="D27" s="9" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="28" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B28" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D28" s="9" t="s">
         <v>55</v>
-      </c>
-      <c r="D28" s="9" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="30" spans="1:5" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
@@ -1836,7 +2243,7 @@
     </row>
     <row r="32" spans="1:5" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="6" t="s">
-        <v>8</v>
+        <v>156</v>
       </c>
       <c r="D32" s="10" t="s">
         <v>5</v>
@@ -1852,7 +2259,7 @@
     </row>
     <row r="34" spans="2:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="6" t="s">
-        <v>10</v>
+        <v>158</v>
       </c>
       <c r="D34" s="10" t="s">
         <v>11</v>
@@ -1868,7 +2275,7 @@
     </row>
     <row r="36" spans="2:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B36" s="6" t="s">
-        <v>10</v>
+        <v>158</v>
       </c>
       <c r="D36" s="10" t="s">
         <v>13</v>
@@ -1886,7 +2293,794 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B49DF9C-BBFA-F34A-9AF2-F8EEB9765D95}">
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="26" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20.1640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="81.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="4.83203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="161.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="10.83203125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="31" x14ac:dyDescent="0.35">
+      <c r="D1" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="31" x14ac:dyDescent="0.35">
+      <c r="D2" s="13"/>
+    </row>
+    <row r="3" spans="1:7" ht="31" x14ac:dyDescent="0.35">
+      <c r="A3" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="13"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="14" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+    </row>
+    <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="11" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+    </row>
+    <row r="12" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" s="4" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+      <c r="B15" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D15" s="20" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C23" s="8"/>
+    </row>
+    <row r="24" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="C24" s="8"/>
+      <c r="D24" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="9" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B27" s="7"/>
+      <c r="C27" s="7"/>
+    </row>
+    <row r="28" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="D29" s="10" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B31" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="D31" s="10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="33" spans="2:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="D33" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D29" r:id="rId1" xr:uid="{7D93EE1F-E819-6049-8956-8F29AF85C45C}"/>
+    <hyperlink ref="D31" r:id="rId2" xr:uid="{031BDA5E-41C4-3E45-9CD9-7CF66935045C}"/>
+    <hyperlink ref="D33" r:id="rId3" xr:uid="{3A2C5DF9-296F-9B4A-B521-4BBA7DFFE365}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C519432A-8521-8343-BFCC-34B0FF74FB19}">
+  <dimension ref="A1:G46"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="26" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20.1640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="77.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="4.83203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="201.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="10.83203125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="31" x14ac:dyDescent="0.35">
+      <c r="D1" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="31" x14ac:dyDescent="0.35">
+      <c r="D2" s="13"/>
+    </row>
+    <row r="3" spans="1:7" ht="31" x14ac:dyDescent="0.35">
+      <c r="A3" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="13"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="14" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+    </row>
+    <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="30" t="s">
+        <v>166</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="30" t="s">
+        <v>162</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="30" t="s">
+        <v>163</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="30" t="s">
+        <v>169</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="30" t="s">
+        <v>170</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="30" t="s">
+        <v>172</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="30" t="s">
+        <v>175</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+    </row>
+    <row r="23" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D24" s="21" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" s="4" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+      <c r="B25" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D25" s="22" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D26" s="21" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D27" s="21" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D28" s="21" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D29" s="21" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" s="4" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+      <c r="B30" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D30" s="22" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B31" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D31" s="21" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D32" s="21" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D33" s="21" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C37" s="8"/>
+    </row>
+    <row r="38" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="9" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B40" s="7"/>
+      <c r="C40" s="7"/>
+    </row>
+    <row r="41" spans="1:7" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B41" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B42" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D42" s="10"/>
+    </row>
+    <row r="43" spans="1:7" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B43" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B44" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D44" s="10"/>
+    </row>
+    <row r="45" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B45" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B46" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="D46" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D46" r:id="rId1" xr:uid="{34BD6D3E-728C-8546-9484-7C8EC6AB0E1D}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{184B1E37-BD29-3B4C-BAA7-E134142B5BF5}">
+  <dimension ref="A1:G39"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="26" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="31.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="87" style="1" customWidth="1"/>
+    <col min="3" max="3" width="4.83203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="201.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" style="1"/>
+    <col min="6" max="6" width="15.83203125" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="10.83203125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="31" x14ac:dyDescent="0.35">
+      <c r="D1" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="31" x14ac:dyDescent="0.35">
+      <c r="D2" s="13"/>
+    </row>
+    <row r="3" spans="1:7" ht="31" x14ac:dyDescent="0.35">
+      <c r="A3" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="13"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="14" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+    </row>
+    <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="9" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="11" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="12" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="13" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="15" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+    </row>
+    <row r="16" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="17" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="D17" s="21"/>
+    </row>
+    <row r="18" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="D18" s="22"/>
+    </row>
+    <row r="19" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="D19" s="21"/>
+    </row>
+    <row r="20" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="D20" s="21" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D21" s="21" t="s">
+        <v>151</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="D22" s="21" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="D23" s="22"/>
+    </row>
+    <row r="24" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="D24" s="21"/>
+    </row>
+    <row r="25" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="D25" s="21"/>
+    </row>
+    <row r="26" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="D26" s="21"/>
+    </row>
+    <row r="27" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="28" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="30" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C30" s="8"/>
+    </row>
+    <row r="31" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="9" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B33" s="7"/>
+      <c r="C33" s="7"/>
+    </row>
+    <row r="34" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D35" s="10" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B36" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B37" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D37" s="10" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B38" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B39" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D39" s="10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D39" r:id="rId1" xr:uid="{3E618234-DA99-934F-B2FA-AE1FBC1B2D72}"/>
+    <hyperlink ref="D35" r:id="rId2" xr:uid="{12ED17EA-24C1-5C49-AB68-FA95BA9C0F84}"/>
+    <hyperlink ref="D37" r:id="rId3" xr:uid="{581D01EC-D486-5140-ABEF-7AC3F113E540}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3606F226-2CE4-CA42-9F8A-8392D3B01B81}">
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="26" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.1640625" style="1" customWidth="1"/>
@@ -1898,511 +3092,205 @@
   <sheetData>
     <row r="1" spans="1:7" ht="31" x14ac:dyDescent="0.35">
       <c r="D1" s="13" t="s">
-        <v>97</v>
+        <v>128</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="31" x14ac:dyDescent="0.35">
       <c r="D2" s="13"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="31" x14ac:dyDescent="0.35">
       <c r="A3" s="11" t="s">
         <v>16</v>
       </c>
+      <c r="D3" s="13"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="12" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
+      <c r="A4" s="14" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-    </row>
-    <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>91</v>
-      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B7" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="10" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
+      <c r="D9" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-    </row>
-    <row r="11" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>94</v>
-      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
     </row>
     <row r="12" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="4" t="s">
-        <v>96</v>
+        <v>137</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>95</v>
+        <v>138</v>
       </c>
     </row>
     <row r="13" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B13" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" s="4" customFormat="1" ht="27" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B14" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="20" t="s">
-        <v>108</v>
+      <c r="D14" s="4" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="15" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B15" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>35</v>
-      </c>
     </row>
     <row r="16" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B16" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D16" s="4" t="s">
-        <v>100</v>
-      </c>
     </row>
     <row r="17" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B17" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D17" s="4" t="s">
-        <v>101</v>
-      </c>
     </row>
     <row r="18" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B18" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D18" s="4" t="s">
-        <v>109</v>
-      </c>
     </row>
     <row r="19" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B19" s="4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="D19" s="4" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>111</v>
-      </c>
+      <c r="C21" s="8"/>
     </row>
     <row r="22" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="C22" s="8"/>
+      <c r="A22" s="9" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="23" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B23" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="C23" s="8"/>
+        <v>127</v>
+      </c>
       <c r="D23" s="9" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="9" t="s">
-        <v>64</v>
-      </c>
+        <v>126</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B25" s="7"/>
+      <c r="C25" s="7"/>
     </row>
     <row r="26" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B26" s="7"/>
-      <c r="C26" s="7"/>
+      <c r="B26" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="27" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>90</v>
+        <v>156</v>
+      </c>
+      <c r="D27" s="10" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="28" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D28" s="10" t="s">
-        <v>89</v>
+        <v>9</v>
       </c>
     </row>
     <row r="29" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" s="10"/>
+    </row>
+    <row r="30" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D29" s="6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D30" s="10" t="s">
-        <v>11</v>
+      <c r="D30" s="6" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="31" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B31" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D32" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="D31" s="10" t="s">
         <v>13</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D28" r:id="rId1" xr:uid="{7D93EE1F-E819-6049-8956-8F29AF85C45C}"/>
-    <hyperlink ref="D30" r:id="rId2" xr:uid="{031BDA5E-41C4-3E45-9CD9-7CF66935045C}"/>
-    <hyperlink ref="D32" r:id="rId3" xr:uid="{3A2C5DF9-296F-9B4A-B521-4BBA7DFFE365}"/>
+    <hyperlink ref="D31" r:id="rId1" xr:uid="{3B0E095A-AF11-974A-9B85-F214E0EB56AE}"/>
+    <hyperlink ref="D27" r:id="rId2" xr:uid="{67F9868B-2DA7-2E47-8970-36214F62A3F9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C519432A-8521-8343-BFCC-34B0FF74FB19}">
-  <dimension ref="A1:G38"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="26" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="20.1640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="72.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.83203125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="201.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="10.83203125" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" ht="31" x14ac:dyDescent="0.35">
-      <c r="D1" s="13" t="s">
-        <v>104</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="31" x14ac:dyDescent="0.35">
-      <c r="D2" s="13"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="11" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="12" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-    </row>
-    <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="11" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="12" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-    </row>
-    <row r="15" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D16" s="21" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" s="4" customFormat="1" ht="27" x14ac:dyDescent="0.3">
-      <c r="B17" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D17" s="22" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D18" s="21" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D19" s="21" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D20" s="21" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D21" s="21" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" s="4" customFormat="1" ht="27" x14ac:dyDescent="0.3">
-      <c r="B22" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D22" s="22" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D23" s="21" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D24" s="21" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D25" s="21" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B29" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="C29" s="8"/>
-    </row>
-    <row r="30" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="9" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B32" s="7"/>
-      <c r="C32" s="7"/>
-    </row>
-    <row r="33" spans="2:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D33" s="6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="34" spans="2:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D34" s="10" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="35" spans="2:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D35" s="6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="36" spans="2:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D36" s="10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="37" spans="2:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D37" s="6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="38" spans="2:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D38" s="10" t="s">
-        <v>13</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="D34" r:id="rId1" xr:uid="{E1B8EF43-7DCA-D748-8F87-A5F7772DD36A}"/>
-    <hyperlink ref="D36" r:id="rId2" xr:uid="{F4C61A5F-10C2-9848-AB81-273A3E47F84D}"/>
-    <hyperlink ref="D38" r:id="rId3" xr:uid="{34BD6D3E-728C-8546-9484-7C8EC6AB0E1D}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9196F1D-D3E3-FA44-AE0F-84C9736C2D9C}">
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="26" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.1640625" style="1" customWidth="1"/>
@@ -2414,203 +3302,221 @@
   <sheetData>
     <row r="1" spans="1:7" ht="31" x14ac:dyDescent="0.35">
       <c r="D1" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>62</v>
-      </c>
     </row>
     <row r="2" spans="1:7" ht="31" x14ac:dyDescent="0.35">
-      <c r="D2" s="13"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D2" s="13" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="31" x14ac:dyDescent="0.35">
       <c r="A3" s="11" t="s">
         <v>16</v>
       </c>
+      <c r="D3" s="13"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="12" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
+      <c r="A4" s="14" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-    </row>
-    <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>32</v>
-      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B7" s="2" t="s">
-        <v>14</v>
+        <v>131</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>17</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
+    </row>
+    <row r="11" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-    </row>
-    <row r="11" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>21</v>
-      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
     </row>
     <row r="12" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
+      </c>
+      <c r="D12" s="26" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B13" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>33</v>
+        <v>29</v>
+      </c>
+      <c r="D13" s="26" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B14" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
+      </c>
+      <c r="D14" s="26" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B15" s="4" t="s">
-        <v>27</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="D15" s="26"/>
     </row>
     <row r="16" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B16" s="4" t="s">
-        <v>28</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="D16" s="26"/>
     </row>
     <row r="17" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B17" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>20</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="D17" s="26"/>
     </row>
     <row r="18" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B18" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D18" s="26" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D19" s="26"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D20" s="25"/>
+    </row>
+    <row r="21" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="C20" s="8"/>
-    </row>
-    <row r="21" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="9" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="7" t="s">
+      <c r="C21" s="8"/>
+      <c r="D21" s="27"/>
+    </row>
+    <row r="22" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="D22" s="27"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D23" s="25"/>
+    </row>
+    <row r="24" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
-    </row>
-    <row r="24" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>4</v>
-      </c>
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="28"/>
     </row>
     <row r="25" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D25" s="10" t="s">
-        <v>5</v>
+        <v>7</v>
+      </c>
+      <c r="D25" s="28" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="26" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="D26" s="29" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="27" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D27" s="28" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D27" s="10" t="s">
+      <c r="D28" s="29" t="s">
         <v>11</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="29" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B29" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D29" s="10" t="s">
+      <c r="D30" s="10" t="s">
         <v>13</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D25" r:id="rId1" xr:uid="{A0D62ABA-3D20-424B-BD68-E17D7BA3EEF2}"/>
-    <hyperlink ref="D27" r:id="rId2" xr:uid="{AECE51C1-FD57-724A-9F2D-14179FC8A173}"/>
-    <hyperlink ref="D29" r:id="rId3" xr:uid="{6BC6D8D5-1D29-D141-B578-F9FD593803D2}"/>
+    <hyperlink ref="D26" r:id="rId1" xr:uid="{A0D62ABA-3D20-424B-BD68-E17D7BA3EEF2}"/>
+    <hyperlink ref="D28" r:id="rId2" xr:uid="{AECE51C1-FD57-724A-9F2D-14179FC8A173}"/>
+    <hyperlink ref="D30" r:id="rId3" xr:uid="{6BC6D8D5-1D29-D141-B578-F9FD593803D2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3606F226-2CE4-CA42-9F8A-8392D3B01B81}">
-  <dimension ref="A1:G29"/>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EAAC078-569D-1D40-BAAF-4BCD49232008}">
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="26" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.1640625" style="1" customWidth="1"/>
@@ -2622,611 +3528,218 @@
   <sheetData>
     <row r="1" spans="1:7" ht="31" x14ac:dyDescent="0.35">
       <c r="D1" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="31" x14ac:dyDescent="0.35">
       <c r="D2" s="13"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="31" x14ac:dyDescent="0.35">
       <c r="A3" s="11" t="s">
         <v>16</v>
       </c>
+      <c r="D3" s="13"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="12" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
+      <c r="A4" s="14" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-    </row>
-    <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>32</v>
-      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="24" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D9" s="24" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D10" s="25"/>
+    </row>
+    <row r="11" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-    </row>
-    <row r="11" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>21</v>
-      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="26"/>
     </row>
     <row r="12" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
+      </c>
+      <c r="D12" s="26" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B13" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>33</v>
+        <v>29</v>
+      </c>
+      <c r="D13" s="26" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B14" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
+      </c>
+      <c r="D14" s="26" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B15" s="4" t="s">
-        <v>27</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="D15" s="26"/>
     </row>
     <row r="16" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B16" s="4" t="s">
-        <v>28</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="D16" s="26"/>
     </row>
     <row r="17" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B17" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>20</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="D17" s="26"/>
     </row>
     <row r="18" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B18" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D18" s="26" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D19" s="26"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D20" s="25"/>
+    </row>
+    <row r="21" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B21" s="8" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="C20" s="8"/>
-    </row>
-    <row r="21" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="9" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="7" t="s">
+      <c r="C21" s="8"/>
+      <c r="D21" s="27"/>
+    </row>
+    <row r="22" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="D22" s="27"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D23" s="25"/>
+    </row>
+    <row r="24" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
-    </row>
-    <row r="24" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>4</v>
-      </c>
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="28"/>
     </row>
     <row r="25" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D25" s="10" t="s">
-        <v>5</v>
+        <v>7</v>
+      </c>
+      <c r="D25" s="28" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="26" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>6</v>
+        <v>8</v>
+      </c>
+      <c r="D26" s="29" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="27" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D27" s="28" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D27" s="10" t="s">
+      <c r="D28" s="29" t="s">
         <v>11</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="29" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B29" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D29" s="10" t="s">
+      <c r="D30" s="10" t="s">
         <v>13</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D25" r:id="rId1" xr:uid="{2CB0D719-28B7-904E-A491-67FC5D52667B}"/>
-    <hyperlink ref="D27" r:id="rId2" xr:uid="{CEAA4B0E-36F3-5849-A615-BCFEC8CF6E36}"/>
-    <hyperlink ref="D29" r:id="rId3" xr:uid="{3B0E095A-AF11-974A-9B85-F214E0EB56AE}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EAAC078-569D-1D40-BAAF-4BCD49232008}">
-  <dimension ref="A1:G29"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="26" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="20.1640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="72.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.83203125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="161.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="10.83203125" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" ht="31" x14ac:dyDescent="0.35">
-      <c r="D1" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="31" x14ac:dyDescent="0.35">
-      <c r="D2" s="13"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="11" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="12" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-    </row>
-    <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-    </row>
-    <row r="11" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="C20" s="8"/>
-    </row>
-    <row r="21" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="9" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
-    </row>
-    <row r="24" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D25" s="10" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D27" s="10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D29" s="10" t="s">
-        <v>13</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="D25" r:id="rId1" xr:uid="{1558357A-BC92-2244-90FB-3EBC102BCA5C}"/>
-    <hyperlink ref="D27" r:id="rId2" xr:uid="{BCDDD629-3CC9-BB43-BD55-529B9E10EFB8}"/>
-    <hyperlink ref="D29" r:id="rId3" xr:uid="{402548E5-623D-5E41-9463-6BCCA88D28E8}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38B8868B-DAAC-D643-93A0-63D9E1CC5FCA}">
-  <dimension ref="A1:G29"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="26" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="20.1640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="72.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.83203125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="161.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="10.83203125" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" ht="31" x14ac:dyDescent="0.35">
-      <c r="D1" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="31" x14ac:dyDescent="0.35">
-      <c r="D2" s="13"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="11" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="12" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-    </row>
-    <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-    </row>
-    <row r="11" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="C20" s="8"/>
-    </row>
-    <row r="21" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="9" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
-    </row>
-    <row r="24" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D25" s="10" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D27" s="10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D29" s="10" t="s">
-        <v>13</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="D25" r:id="rId1" xr:uid="{0AA4F660-30A1-BF4B-9DA6-F38F3FB6789B}"/>
-    <hyperlink ref="D27" r:id="rId2" xr:uid="{407F8995-E5CF-F840-9500-E41EF8A0727D}"/>
-    <hyperlink ref="D29" r:id="rId3" xr:uid="{3B0FA85A-A8DF-6D4D-BD35-F91776B09DDE}"/>
+    <hyperlink ref="D26" r:id="rId1" xr:uid="{1558357A-BC92-2244-90FB-3EBC102BCA5C}"/>
+    <hyperlink ref="D28" r:id="rId2" xr:uid="{BCDDD629-3CC9-BB43-BD55-529B9E10EFB8}"/>
+    <hyperlink ref="D30" r:id="rId3" xr:uid="{402548E5-623D-5E41-9463-6BCCA88D28E8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updating QIAL data tracker (Hanwen\'s columns).
</commit_message>
<xml_diff>
--- a/QIAL_data_tracker_2019_2026.xlsx
+++ b/QIAL_data_tracker_2019_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rja20/Documents/MATLAB/gunnies/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jas/Documents/MATLAB/gunnies/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E76E5F50-72B5-B24F-80CC-3E0BD64EDB59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BE92BE8-7655-C84C-86C2-680349AC7029}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11120" yWindow="4780" windowWidth="38460" windowHeight="20300" activeTab="4" xr2:uid="{BEE67711-3DDE-B344-B789-C2167E37D311}"/>
+    <workbookView xWindow="3880" yWindow="1420" windowWidth="45560" windowHeight="20820" activeTab="1" xr2:uid="{BEE67711-3DDE-B344-B789-C2167E37D311}"/>
   </bookViews>
   <sheets>
     <sheet name="ADRC_human" sheetId="2" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="181">
   <si>
     <t>Raw Data</t>
   </si>
@@ -293,9 +293,6 @@
     <t>$WORK/hanwen/ad_decode_test/input/S*/</t>
   </si>
   <si>
-    <t>Hanwen's Columns</t>
-  </si>
-  <si>
     <t>Hanwen's Thicknesses</t>
   </si>
   <si>
@@ -594,6 +591,15 @@
   </si>
   <si>
     <t>Raw niftis, btables:</t>
+  </si>
+  <si>
+    <t>$WORK/hanwen/ad_decode_test/output/S*/QSM/</t>
+  </si>
+  <si>
+    <t>Hanwen's Columns (QSM)</t>
+  </si>
+  <si>
+    <t>Hanwen's Columns (except QSM)</t>
   </si>
 </sst>
 </file>
@@ -787,7 +793,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -825,6 +831,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -850,9 +857,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -890,7 +897,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -996,7 +1003,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1138,7 +1145,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1231,7 +1238,7 @@
         <v>23</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="13" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -1247,7 +1254,7 @@
         <v>25</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="15" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -1279,7 +1286,7 @@
         <v>22</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="19" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -1350,7 +1357,7 @@
     </row>
     <row r="30" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B30" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D30" s="10" t="s">
         <v>13</v>
@@ -1380,7 +1387,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="31" x14ac:dyDescent="0.35">
       <c r="D1" s="13" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>58</v>
@@ -1599,7 +1606,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B3C5125-DEBE-914D-B850-27AB6E3ABDEE}">
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23.6640625" customWidth="1"/>
@@ -1704,7 +1711,7 @@
     <row r="10" spans="1:7" s="17" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
       <c r="B10" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2" t="s">
@@ -1750,7 +1757,7 @@
     <row r="14" spans="1:7" ht="26" x14ac:dyDescent="0.3">
       <c r="A14" s="4"/>
       <c r="B14" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C14" s="4"/>
       <c r="D14" s="4" t="s">
@@ -1763,11 +1770,11 @@
     <row r="15" spans="1:7" ht="26" x14ac:dyDescent="0.3">
       <c r="A15" s="18"/>
       <c r="B15" s="18" t="s">
-        <v>78</v>
+        <v>180</v>
       </c>
       <c r="C15" s="18"/>
       <c r="D15" s="18" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E15" s="18"/>
       <c r="F15" s="18"/>
@@ -1776,50 +1783,50 @@
     <row r="16" spans="1:7" s="17" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A16" s="4"/>
       <c r="B16" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C16" s="4"/>
       <c r="D16" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
     </row>
-    <row r="17" spans="1:7" ht="26" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" s="31" customFormat="1" ht="26" x14ac:dyDescent="0.3">
       <c r="A17" s="19"/>
       <c r="B17" s="19" t="s">
-        <v>29</v>
+        <v>179</v>
       </c>
       <c r="C17" s="19"/>
       <c r="D17" s="19" t="s">
-        <v>106</v>
+        <v>178</v>
       </c>
       <c r="E17" s="19"/>
       <c r="F17" s="19"/>
       <c r="G17" s="19"/>
     </row>
     <row r="18" spans="1:7" ht="26" x14ac:dyDescent="0.3">
-      <c r="A18" s="4"/>
-      <c r="B18" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="23" t="s">
-        <v>107</v>
-      </c>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
+      <c r="A18" s="19"/>
+      <c r="B18" s="19" t="s">
+        <v>29</v>
+      </c>
+      <c r="C18" s="19"/>
+      <c r="D18" s="19" t="s">
+        <v>105</v>
+      </c>
+      <c r="E18" s="19"/>
+      <c r="F18" s="19"/>
+      <c r="G18" s="19"/>
     </row>
     <row r="19" spans="1:7" ht="26" x14ac:dyDescent="0.3">
       <c r="A19" s="4"/>
       <c r="B19" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C19" s="4"/>
-      <c r="D19" s="21" t="s">
-        <v>34</v>
+      <c r="D19" s="23" t="s">
+        <v>106</v>
       </c>
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
@@ -1828,11 +1835,11 @@
     <row r="20" spans="1:7" ht="26" x14ac:dyDescent="0.3">
       <c r="A20" s="4"/>
       <c r="B20" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C20" s="4"/>
       <c r="D20" s="21" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
@@ -1841,11 +1848,11 @@
     <row r="21" spans="1:7" ht="26" x14ac:dyDescent="0.3">
       <c r="A21" s="4"/>
       <c r="B21" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C21" s="4"/>
       <c r="D21" s="21" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
@@ -1854,11 +1861,11 @@
     <row r="22" spans="1:7" ht="26" x14ac:dyDescent="0.3">
       <c r="A22" s="4"/>
       <c r="B22" s="4" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C22" s="4"/>
-      <c r="D22" s="4" t="s">
-        <v>86</v>
+      <c r="D22" s="21" t="s">
+        <v>36</v>
       </c>
       <c r="E22" s="4"/>
       <c r="F22" s="4"/>
@@ -1866,88 +1873,88 @@
     </row>
     <row r="23" spans="1:7" ht="26" x14ac:dyDescent="0.3">
       <c r="A23" s="4"/>
-      <c r="B23" s="4"/>
+      <c r="B23" s="4" t="s">
+        <v>22</v>
+      </c>
       <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
+      <c r="D23" s="4" t="s">
+        <v>85</v>
+      </c>
       <c r="E23" s="4"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
     </row>
     <row r="24" spans="1:7" ht="26" x14ac:dyDescent="0.3">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
+      <c r="A24" s="4"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+      <c r="G24" s="4"/>
     </row>
     <row r="25" spans="1:7" ht="26" x14ac:dyDescent="0.3">
-      <c r="A25" s="8" t="s">
+      <c r="A25" s="1"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
+    </row>
+    <row r="26" spans="1:7" ht="26" x14ac:dyDescent="0.3">
+      <c r="A26" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B26" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="C25" s="8"/>
-      <c r="D25" s="9"/>
-      <c r="E25" s="9"/>
-      <c r="F25" s="9"/>
-      <c r="G25" s="9"/>
-    </row>
-    <row r="26" spans="1:7" ht="26" x14ac:dyDescent="0.3">
-      <c r="A26" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="B26" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9" t="s">
-        <v>84</v>
-      </c>
+      <c r="C26" s="8"/>
+      <c r="D26" s="9"/>
       <c r="E26" s="9"/>
       <c r="F26" s="9"/>
       <c r="G26" s="9"/>
     </row>
     <row r="27" spans="1:7" ht="26" x14ac:dyDescent="0.3">
-      <c r="A27" s="15"/>
-      <c r="B27" s="15"/>
-      <c r="C27" s="15"/>
-      <c r="D27" s="15"/>
-      <c r="E27" s="15"/>
-      <c r="F27" s="15"/>
-      <c r="G27" s="15"/>
+      <c r="A27" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
     </row>
     <row r="28" spans="1:7" ht="26" x14ac:dyDescent="0.3">
-      <c r="A28" s="1"/>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
-      <c r="E28" s="1"/>
-      <c r="F28" s="1"/>
-      <c r="G28" s="1"/>
+      <c r="A28" s="15"/>
+      <c r="B28" s="15"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
     </row>
     <row r="29" spans="1:7" ht="26" x14ac:dyDescent="0.3">
-      <c r="A29" s="7" t="s">
+      <c r="A29" s="1"/>
+      <c r="B29" s="1"/>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+    </row>
+    <row r="30" spans="1:7" ht="26" x14ac:dyDescent="0.3">
+      <c r="A30" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B29" s="7"/>
-      <c r="C29" s="7"/>
-      <c r="D29" s="6"/>
-      <c r="E29" s="6"/>
-      <c r="F29" s="6"/>
-      <c r="G29" s="6"/>
-    </row>
-    <row r="30" spans="1:7" ht="26" x14ac:dyDescent="0.3">
-      <c r="A30" s="6"/>
-      <c r="B30" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C30" s="6"/>
-      <c r="D30" s="6" t="s">
-        <v>4</v>
-      </c>
+      <c r="B30" s="7"/>
+      <c r="C30" s="7"/>
+      <c r="D30" s="6"/>
       <c r="E30" s="6"/>
       <c r="F30" s="6"/>
       <c r="G30" s="6"/>
@@ -1955,11 +1962,11 @@
     <row r="31" spans="1:7" ht="26" x14ac:dyDescent="0.3">
       <c r="A31" s="6"/>
       <c r="B31" s="6" t="s">
-        <v>156</v>
+        <v>7</v>
       </c>
       <c r="C31" s="6"/>
-      <c r="D31" s="10" t="s">
-        <v>5</v>
+      <c r="D31" s="6" t="s">
+        <v>4</v>
       </c>
       <c r="E31" s="6"/>
       <c r="F31" s="6"/>
@@ -1968,11 +1975,11 @@
     <row r="32" spans="1:7" ht="26" x14ac:dyDescent="0.3">
       <c r="A32" s="6"/>
       <c r="B32" s="6" t="s">
-        <v>9</v>
+        <v>155</v>
       </c>
       <c r="C32" s="6"/>
-      <c r="D32" s="6" t="s">
-        <v>6</v>
+      <c r="D32" s="10" t="s">
+        <v>5</v>
       </c>
       <c r="E32" s="6"/>
       <c r="F32" s="6"/>
@@ -1981,11 +1988,11 @@
     <row r="33" spans="1:7" ht="26" x14ac:dyDescent="0.3">
       <c r="A33" s="6"/>
       <c r="B33" s="6" t="s">
-        <v>158</v>
+        <v>9</v>
       </c>
       <c r="C33" s="6"/>
-      <c r="D33" s="10" t="s">
-        <v>11</v>
+      <c r="D33" s="6" t="s">
+        <v>6</v>
       </c>
       <c r="E33" s="6"/>
       <c r="F33" s="6"/>
@@ -1994,11 +2001,11 @@
     <row r="34" spans="1:7" ht="26" x14ac:dyDescent="0.3">
       <c r="A34" s="6"/>
       <c r="B34" s="6" t="s">
-        <v>9</v>
+        <v>157</v>
       </c>
       <c r="C34" s="6"/>
-      <c r="D34" s="6" t="s">
-        <v>12</v>
+      <c r="D34" s="10" t="s">
+        <v>11</v>
       </c>
       <c r="E34" s="6"/>
       <c r="F34" s="6"/>
@@ -2007,21 +2014,34 @@
     <row r="35" spans="1:7" ht="26" x14ac:dyDescent="0.3">
       <c r="A35" s="6"/>
       <c r="B35" s="6" t="s">
-        <v>158</v>
+        <v>9</v>
       </c>
       <c r="C35" s="6"/>
-      <c r="D35" s="10" t="s">
-        <v>13</v>
+      <c r="D35" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="E35" s="6"/>
       <c r="F35" s="6"/>
       <c r="G35" s="6"/>
     </row>
+    <row r="36" spans="1:7" ht="26" x14ac:dyDescent="0.3">
+      <c r="A36" s="6"/>
+      <c r="B36" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="C36" s="6"/>
+      <c r="D36" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E36" s="6"/>
+      <c r="F36" s="6"/>
+      <c r="G36" s="6"/>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D31" r:id="rId1" xr:uid="{A881BDA2-E667-3F49-AE16-C91CBE79A2FA}"/>
-    <hyperlink ref="D33" r:id="rId2" xr:uid="{CD718C81-2310-2F44-8928-FF24A7358A14}"/>
-    <hyperlink ref="D35" r:id="rId3" xr:uid="{8F4E9AED-317C-BC4E-8FD6-5EB8D63BE6DF}"/>
+    <hyperlink ref="D32" r:id="rId1" xr:uid="{A881BDA2-E667-3F49-AE16-C91CBE79A2FA}"/>
+    <hyperlink ref="D34" r:id="rId2" xr:uid="{CD718C81-2310-2F44-8928-FF24A7358A14}"/>
+    <hyperlink ref="D36" r:id="rId3" xr:uid="{8F4E9AED-317C-BC4E-8FD6-5EB8D63BE6DF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -2126,7 +2146,7 @@
         <v>25</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2243,7 +2263,7 @@
     </row>
     <row r="32" spans="1:5" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D32" s="10" t="s">
         <v>5</v>
@@ -2259,7 +2279,7 @@
     </row>
     <row r="34" spans="2:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D34" s="10" t="s">
         <v>11</v>
@@ -2275,7 +2295,7 @@
     </row>
     <row r="36" spans="2:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B36" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D36" s="10" t="s">
         <v>13</v>
@@ -2305,7 +2325,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="31" x14ac:dyDescent="0.35">
       <c r="D1" s="13" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>58</v>
@@ -2345,10 +2365,10 @@
     </row>
     <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B7" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -2356,7 +2376,7 @@
         <v>18</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="9" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3"/>
@@ -2372,15 +2392,15 @@
         <v>23</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="13" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B13" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2388,7 +2408,7 @@
         <v>29</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:7" s="4" customFormat="1" ht="27" x14ac:dyDescent="0.3">
@@ -2396,7 +2416,7 @@
         <v>25</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="16" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2412,7 +2432,7 @@
         <v>27</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="18" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2420,7 +2440,7 @@
         <v>28</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="19" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2428,7 +2448,7 @@
         <v>22</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="20" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2436,7 +2456,7 @@
         <v>56</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="21" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2444,7 +2464,7 @@
         <v>46</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="23" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
@@ -2462,7 +2482,7 @@
       </c>
       <c r="C24" s="8"/>
       <c r="D24" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="25" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
@@ -2482,15 +2502,15 @@
         <v>7</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="29" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="30" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
@@ -2503,7 +2523,7 @@
     </row>
     <row r="31" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D31" s="10" t="s">
         <v>11</v>
@@ -2519,7 +2539,7 @@
     </row>
     <row r="33" spans="2:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B33" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D33" s="10" t="s">
         <v>13</v>
@@ -2549,7 +2569,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="31" x14ac:dyDescent="0.35">
       <c r="D1" s="13" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>58</v>
@@ -2589,114 +2609,114 @@
     </row>
     <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B8" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B9" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>114</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="10" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="11" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B11" s="30" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="12" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="30" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="13" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B13" s="30" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="14" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B14" s="30" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="15" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B15" s="30" t="s">
+        <v>169</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>170</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="16" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B16" s="30" t="s">
+        <v>171</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>172</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="17" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B17" s="30" t="s">
+        <v>174</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>175</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>176</v>
       </c>
     </row>
     <row r="18" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B18" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="19" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="20" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B20" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="22" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2716,13 +2736,13 @@
     </row>
     <row r="24" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>29</v>
       </c>
       <c r="D24" s="21" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="25" spans="1:4" s="4" customFormat="1" ht="27" x14ac:dyDescent="0.3">
@@ -2730,7 +2750,7 @@
         <v>25</v>
       </c>
       <c r="D25" s="22" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="26" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2746,7 +2766,7 @@
         <v>27</v>
       </c>
       <c r="D27" s="21" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="28" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2754,18 +2774,18 @@
         <v>28</v>
       </c>
       <c r="D28" s="21" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="29" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>29</v>
       </c>
       <c r="D29" s="21" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="30" spans="1:4" s="4" customFormat="1" ht="27" x14ac:dyDescent="0.3">
@@ -2773,7 +2793,7 @@
         <v>25</v>
       </c>
       <c r="D30" s="22" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="31" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2789,7 +2809,7 @@
         <v>27</v>
       </c>
       <c r="D32" s="21" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="33" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2797,7 +2817,7 @@
         <v>28</v>
       </c>
       <c r="D33" s="21" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="34" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2805,7 +2825,7 @@
         <v>22</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="35" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -2866,7 +2886,7 @@
     </row>
     <row r="46" spans="1:7" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B46" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D46" s="10" t="s">
         <v>13</v>
@@ -2896,7 +2916,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="31" x14ac:dyDescent="0.35">
       <c r="D1" s="13" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>58</v>
@@ -2957,38 +2977,38 @@
     </row>
     <row r="19" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D19" s="21"/>
     </row>
     <row r="20" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="D20" s="21" t="s">
         <v>145</v>
-      </c>
-      <c r="D20" s="21" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="21" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B21" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="D21" s="21" t="s">
         <v>150</v>
       </c>
-      <c r="D21" s="21" t="s">
+      <c r="F21" s="4" t="s">
         <v>151</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="22" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B22" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D22" s="21" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="23" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -3036,7 +3056,7 @@
         <v>8</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="36" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
@@ -3049,12 +3069,12 @@
         <v>10</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="38" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B38" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D38" s="6" t="s">
         <v>12</v>
@@ -3092,7 +3112,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="31" x14ac:dyDescent="0.35">
       <c r="D1" s="13" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>58</v>
@@ -3132,10 +3152,10 @@
     </row>
     <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B7" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -3143,7 +3163,7 @@
         <v>14</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="9" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -3151,7 +3171,7 @@
         <v>18</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="11" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -3163,10 +3183,10 @@
     </row>
     <row r="12" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B12" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>137</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="13" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -3179,7 +3199,7 @@
         <v>25</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="15" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
@@ -3204,7 +3224,7 @@
     </row>
     <row r="19" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B19" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="21" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
@@ -3223,10 +3243,10 @@
     </row>
     <row r="23" spans="1:4" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B23" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="25" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
@@ -3241,15 +3261,15 @@
         <v>7</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="27" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="28" spans="1:4" s="6" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.3">
@@ -3273,7 +3293,7 @@
     </row>
     <row r="31" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B31" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D31" s="10" t="s">
         <v>13</v>
@@ -3302,7 +3322,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="31" x14ac:dyDescent="0.35">
       <c r="D1" s="13" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>58</v>
@@ -3316,7 +3336,7 @@
     </row>
     <row r="2" spans="1:7" ht="31" x14ac:dyDescent="0.35">
       <c r="D2" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="31" x14ac:dyDescent="0.35">
@@ -3344,10 +3364,10 @@
     </row>
     <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B7" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -3355,7 +3375,7 @@
         <v>14</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.3">
@@ -3528,7 +3548,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="31" x14ac:dyDescent="0.35">
       <c r="D1" s="13" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>58</v>

</xml_diff>